<commit_message>
change plot range from 6 to 9
</commit_message>
<xml_diff>
--- a/Groundtruth/roi_coordinates2.xlsx
+++ b/Groundtruth/roi_coordinates2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hosse\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VIS2025\BIoVisChallenges\SSGAT\Groundtruth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0DCF4B4-7F1F-44B5-BBD6-033D82AD9423}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E54B9B1B-CAB0-4B28-96C3-FCA7FD74A9B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="T-cell_maturation" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="16">
   <si>
     <t>ROI_ID</t>
   </si>
@@ -63,12 +63,21 @@
   <si>
     <t>GAY</t>
   </si>
+  <si>
+    <t>Person 7</t>
+  </si>
+  <si>
+    <t>Person 8</t>
+  </si>
+  <si>
+    <t>Person 9</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -81,6 +90,12 @@
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -90,7 +105,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -128,16 +143,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -442,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -844,7 +876,7 @@
         <v>3</v>
       </c>
       <c r="C24" s="2">
-        <v>4990</v>
+        <v>6790</v>
       </c>
       <c r="D24" s="2">
         <v>2850</v>
@@ -918,7 +950,7 @@
         <v>865</v>
       </c>
       <c r="E28" s="2">
-        <v>155</v>
+        <v>105</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -929,10 +961,10 @@
         <v>3</v>
       </c>
       <c r="C29" s="2">
-        <v>7887</v>
+        <v>8100</v>
       </c>
       <c r="D29" s="2">
-        <v>3194</v>
+        <v>3094</v>
       </c>
       <c r="E29" s="2">
         <v>50</v>
@@ -963,10 +995,10 @@
         <v>5</v>
       </c>
       <c r="C31" s="2">
-        <v>2187</v>
+        <v>2387</v>
       </c>
       <c r="D31" s="2">
-        <v>2049</v>
+        <v>1249</v>
       </c>
       <c r="E31" s="2">
         <v>75</v>
@@ -997,10 +1029,10 @@
         <v>2</v>
       </c>
       <c r="C33" s="2">
+        <v>2100</v>
+      </c>
+      <c r="D33" s="2">
         <v>1330</v>
-      </c>
-      <c r="D33" s="2">
-        <v>2127</v>
       </c>
       <c r="E33" s="2">
         <v>34</v>
@@ -1014,7 +1046,7 @@
         <v>3</v>
       </c>
       <c r="C34" s="2">
-        <v>4976</v>
+        <v>8976</v>
       </c>
       <c r="D34" s="2">
         <v>3019</v>
@@ -1031,13 +1063,13 @@
         <v>4</v>
       </c>
       <c r="C35" s="2">
-        <v>9055</v>
+        <v>4835</v>
       </c>
       <c r="D35" s="2">
-        <v>3950</v>
+        <v>4327</v>
       </c>
       <c r="E35" s="2">
-        <v>145</v>
+        <v>162</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
@@ -1048,23 +1080,279 @@
         <v>5</v>
       </c>
       <c r="C36" s="2">
-        <v>4835</v>
+        <v>9555</v>
       </c>
       <c r="D36" s="2">
-        <v>4327</v>
+        <v>4750</v>
       </c>
       <c r="E36" s="2">
-        <v>162</v>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="2">
+        <v>1</v>
+      </c>
+      <c r="C37" s="3">
+        <v>808</v>
+      </c>
+      <c r="D37" s="3">
+        <v>970</v>
+      </c>
+      <c r="E37" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" s="2">
+        <v>2</v>
+      </c>
+      <c r="C38" s="3">
+        <v>2610</v>
+      </c>
+      <c r="D38" s="3">
+        <v>1320</v>
+      </c>
+      <c r="E38" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B39" s="2">
+        <v>3</v>
+      </c>
+      <c r="C39" s="3">
+        <v>5980</v>
+      </c>
+      <c r="D39" s="3">
+        <v>2779</v>
+      </c>
+      <c r="E39" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" s="2">
+        <v>4</v>
+      </c>
+      <c r="C40" s="3">
+        <v>8490</v>
+      </c>
+      <c r="D40" s="3">
+        <v>3376</v>
+      </c>
+      <c r="E40" s="3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" s="2">
+        <v>5</v>
+      </c>
+      <c r="C41" s="3">
+        <v>9440</v>
+      </c>
+      <c r="D41" s="3">
+        <v>4600</v>
+      </c>
+      <c r="E41" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" s="2">
+        <v>1</v>
+      </c>
+      <c r="C42" s="3">
+        <v>500</v>
+      </c>
+      <c r="D42" s="3">
+        <v>900</v>
+      </c>
+      <c r="E42" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" s="2">
+        <v>2</v>
+      </c>
+      <c r="C43" s="3">
+        <v>6394</v>
+      </c>
+      <c r="D43" s="3">
+        <v>2872</v>
+      </c>
+      <c r="E43" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44" s="2">
+        <v>3</v>
+      </c>
+      <c r="C44" s="3">
+        <v>8777</v>
+      </c>
+      <c r="D44" s="3">
+        <v>3217</v>
+      </c>
+      <c r="E44" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B45" s="2">
+        <v>4</v>
+      </c>
+      <c r="C45" s="3">
+        <v>9828</v>
+      </c>
+      <c r="D45" s="3">
+        <v>4625</v>
+      </c>
+      <c r="E45" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B46" s="2">
+        <v>5</v>
+      </c>
+      <c r="C46" s="3">
+        <v>6132</v>
+      </c>
+      <c r="D46" s="3">
+        <v>3044</v>
+      </c>
+      <c r="E46" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="2">
+        <v>1</v>
+      </c>
+      <c r="C47" s="3">
+        <v>9890</v>
+      </c>
+      <c r="D47" s="3">
+        <v>4390</v>
+      </c>
+      <c r="E47" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B48" s="2">
+        <v>2</v>
+      </c>
+      <c r="C48" s="3">
+        <v>500</v>
+      </c>
+      <c r="D48" s="3">
+        <v>880</v>
+      </c>
+      <c r="E48" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B49" s="2">
+        <v>3</v>
+      </c>
+      <c r="C49" s="3">
+        <v>6354</v>
+      </c>
+      <c r="D49" s="3">
+        <v>2708</v>
+      </c>
+      <c r="E49" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B50" s="2">
+        <v>4</v>
+      </c>
+      <c r="C50" s="3">
+        <v>8500</v>
+      </c>
+      <c r="D50" s="3">
+        <v>3290</v>
+      </c>
+      <c r="E50" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B51" s="2">
+        <v>5</v>
+      </c>
+      <c r="C51" s="3">
+        <v>900</v>
+      </c>
+      <c r="D51" s="3">
+        <v>1100</v>
+      </c>
+      <c r="E51" s="3">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -1098,7 +1386,7 @@
         <v>384</v>
       </c>
       <c r="E2">
-        <v>0</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -1677,6 +1965,261 @@
       </c>
       <c r="E36" s="2">
         <v>161</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="2">
+        <v>1</v>
+      </c>
+      <c r="C37" s="3">
+        <v>1090</v>
+      </c>
+      <c r="D37" s="3">
+        <v>1040</v>
+      </c>
+      <c r="E37" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" s="2">
+        <v>2</v>
+      </c>
+      <c r="C38" s="3">
+        <v>2514</v>
+      </c>
+      <c r="D38" s="3">
+        <v>1950</v>
+      </c>
+      <c r="E38" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B39" s="2">
+        <v>3</v>
+      </c>
+      <c r="C39" s="3">
+        <v>3114</v>
+      </c>
+      <c r="D39" s="3">
+        <v>2142</v>
+      </c>
+      <c r="E39" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" s="2">
+        <v>4</v>
+      </c>
+      <c r="C40" s="3">
+        <v>8200</v>
+      </c>
+      <c r="D40" s="3">
+        <v>3900</v>
+      </c>
+      <c r="E40" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" s="2">
+        <v>5</v>
+      </c>
+      <c r="C41" s="3">
+        <v>9000</v>
+      </c>
+      <c r="D41" s="3">
+        <v>3400</v>
+      </c>
+      <c r="E41" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" s="2">
+        <v>1</v>
+      </c>
+      <c r="C42" s="3">
+        <v>807</v>
+      </c>
+      <c r="D42" s="3">
+        <v>721</v>
+      </c>
+      <c r="E42" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" s="2">
+        <v>2</v>
+      </c>
+      <c r="C43" s="3">
+        <v>2300</v>
+      </c>
+      <c r="D43" s="3">
+        <v>1900</v>
+      </c>
+      <c r="E43" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44" s="2">
+        <v>3</v>
+      </c>
+      <c r="C44" s="3">
+        <v>8772</v>
+      </c>
+      <c r="D44" s="3">
+        <v>3141</v>
+      </c>
+      <c r="E44" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B45" s="2">
+        <v>4</v>
+      </c>
+      <c r="C45" s="3">
+        <v>6304</v>
+      </c>
+      <c r="D45" s="3">
+        <v>3202</v>
+      </c>
+      <c r="E45" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B46" s="2">
+        <v>5</v>
+      </c>
+      <c r="C46" s="3">
+        <v>3200</v>
+      </c>
+      <c r="D46" s="3">
+        <v>1900</v>
+      </c>
+      <c r="E46" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="2">
+        <v>1</v>
+      </c>
+      <c r="C47" s="3">
+        <v>8736</v>
+      </c>
+      <c r="D47" s="3">
+        <v>3217</v>
+      </c>
+      <c r="E47" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B48" s="2">
+        <v>2</v>
+      </c>
+      <c r="C48" s="3">
+        <v>9041</v>
+      </c>
+      <c r="D48" s="3">
+        <v>3600</v>
+      </c>
+      <c r="E48" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B49" s="2">
+        <v>3</v>
+      </c>
+      <c r="C49" s="3">
+        <v>2403</v>
+      </c>
+      <c r="D49" s="3">
+        <v>2307</v>
+      </c>
+      <c r="E49" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B50" s="2">
+        <v>4</v>
+      </c>
+      <c r="C50" s="3">
+        <v>946</v>
+      </c>
+      <c r="D50" s="3">
+        <v>1208</v>
+      </c>
+      <c r="E50" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B51" s="2">
+        <v>5</v>
+      </c>
+      <c r="C51" s="3">
+        <v>591</v>
+      </c>
+      <c r="D51" s="3">
+        <v>389</v>
+      </c>
+      <c r="E51" s="3">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -1686,7 +2229,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -1884,10 +2427,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="2">
-        <v>780</v>
+        <v>480</v>
       </c>
       <c r="D12" s="2">
-        <v>2313</v>
+        <v>313</v>
       </c>
       <c r="E12" s="2">
         <v>96</v>
@@ -1901,10 +2444,10 @@
         <v>2</v>
       </c>
       <c r="C13" s="2">
-        <v>7001</v>
+        <v>701</v>
       </c>
       <c r="D13" s="2">
-        <v>2150</v>
+        <v>1150</v>
       </c>
       <c r="E13" s="2">
         <v>96</v>
@@ -2190,10 +2733,10 @@
         <v>4</v>
       </c>
       <c r="C30" s="2">
-        <v>9637</v>
+        <v>9837</v>
       </c>
       <c r="D30" s="2">
-        <v>3139</v>
+        <v>4739</v>
       </c>
       <c r="E30" s="2">
         <v>118</v>
@@ -2207,10 +2750,10 @@
         <v>5</v>
       </c>
       <c r="C31" s="2">
-        <v>6214</v>
+        <v>5914</v>
       </c>
       <c r="D31" s="2">
-        <v>4363</v>
+        <v>3363</v>
       </c>
       <c r="E31" s="2">
         <v>158</v>
@@ -2241,10 +2784,10 @@
         <v>2</v>
       </c>
       <c r="C33" s="2">
-        <v>865</v>
+        <v>665</v>
       </c>
       <c r="D33" s="2">
-        <v>1700</v>
+        <v>1024</v>
       </c>
       <c r="E33" s="2">
         <v>48</v>
@@ -2258,10 +2801,10 @@
         <v>3</v>
       </c>
       <c r="C34" s="2">
-        <v>9015</v>
+        <v>9915</v>
       </c>
       <c r="D34" s="2">
-        <v>3020</v>
+        <v>4820</v>
       </c>
       <c r="E34" s="2">
         <v>43</v>
@@ -2275,10 +2818,10 @@
         <v>4</v>
       </c>
       <c r="C35" s="2">
-        <v>5400</v>
+        <v>5815</v>
       </c>
       <c r="D35" s="2">
-        <v>2400</v>
+        <v>3432</v>
       </c>
       <c r="E35" s="2">
         <v>104</v>
@@ -2292,13 +2835,268 @@
         <v>5</v>
       </c>
       <c r="C36" s="2">
-        <v>3698</v>
+        <v>9698</v>
       </c>
       <c r="D36" s="2">
-        <v>688</v>
+        <v>4688</v>
       </c>
       <c r="E36" s="2">
         <v>160</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="2">
+        <v>1</v>
+      </c>
+      <c r="C37" s="3">
+        <v>350</v>
+      </c>
+      <c r="D37" s="3">
+        <v>430</v>
+      </c>
+      <c r="E37" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" s="2">
+        <v>2</v>
+      </c>
+      <c r="C38" s="3">
+        <v>650</v>
+      </c>
+      <c r="D38" s="3">
+        <v>1054</v>
+      </c>
+      <c r="E38" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B39" s="2">
+        <v>3</v>
+      </c>
+      <c r="C39" s="3">
+        <v>2504</v>
+      </c>
+      <c r="D39" s="3">
+        <v>2100</v>
+      </c>
+      <c r="E39" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" s="2">
+        <v>4</v>
+      </c>
+      <c r="C40" s="3">
+        <v>5690</v>
+      </c>
+      <c r="D40" s="3">
+        <v>3394</v>
+      </c>
+      <c r="E40" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" s="2">
+        <v>5</v>
+      </c>
+      <c r="C41" s="3">
+        <v>7950</v>
+      </c>
+      <c r="D41" s="3">
+        <v>4028</v>
+      </c>
+      <c r="E41" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" s="2">
+        <v>1</v>
+      </c>
+      <c r="C42" s="3">
+        <v>730</v>
+      </c>
+      <c r="D42" s="3">
+        <v>810</v>
+      </c>
+      <c r="E42" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" s="2">
+        <v>2</v>
+      </c>
+      <c r="C43" s="3">
+        <v>2018</v>
+      </c>
+      <c r="D43" s="3">
+        <v>1950</v>
+      </c>
+      <c r="E43" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44" s="2">
+        <v>3</v>
+      </c>
+      <c r="C44" s="3">
+        <v>5850</v>
+      </c>
+      <c r="D44" s="3">
+        <v>3561</v>
+      </c>
+      <c r="E44" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B45" s="2">
+        <v>4</v>
+      </c>
+      <c r="C45" s="3">
+        <v>4561</v>
+      </c>
+      <c r="D45" s="3">
+        <v>2480</v>
+      </c>
+      <c r="E45" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B46" s="2">
+        <v>5</v>
+      </c>
+      <c r="C46" s="3">
+        <v>10168</v>
+      </c>
+      <c r="D46" s="3">
+        <v>4594</v>
+      </c>
+      <c r="E46" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="2">
+        <v>1</v>
+      </c>
+      <c r="C47" s="3">
+        <v>730</v>
+      </c>
+      <c r="D47" s="3">
+        <v>850</v>
+      </c>
+      <c r="E47" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B48" s="2">
+        <v>2</v>
+      </c>
+      <c r="C48" s="3">
+        <v>9892</v>
+      </c>
+      <c r="D48" s="3">
+        <v>4582</v>
+      </c>
+      <c r="E48" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B49" s="2">
+        <v>3</v>
+      </c>
+      <c r="C49" s="3">
+        <v>2421</v>
+      </c>
+      <c r="D49" s="3">
+        <v>2152</v>
+      </c>
+      <c r="E49" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B50" s="2">
+        <v>4</v>
+      </c>
+      <c r="C50" s="3">
+        <v>2005</v>
+      </c>
+      <c r="D50" s="3">
+        <v>1150</v>
+      </c>
+      <c r="E50" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B51" s="2">
+        <v>5</v>
+      </c>
+      <c r="C51" s="4">
+        <v>591</v>
+      </c>
+      <c r="D51" s="4">
+        <v>432</v>
+      </c>
+      <c r="E51" s="4">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2308,7 +3106,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -2421,7 +3219,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="2">
-        <v>8593</v>
+        <v>7952</v>
       </c>
       <c r="D7" s="2">
         <v>3251</v>
@@ -2438,10 +3236,10 @@
         <v>2</v>
       </c>
       <c r="C8" s="2">
-        <v>9719</v>
+        <v>6519</v>
       </c>
       <c r="D8" s="2">
-        <v>3900</v>
+        <v>2315</v>
       </c>
       <c r="E8" s="2">
         <v>85</v>
@@ -2458,7 +3256,7 @@
         <v>129</v>
       </c>
       <c r="D9" s="2">
-        <v>1700</v>
+        <v>1680</v>
       </c>
       <c r="E9" s="2">
         <v>159</v>
@@ -2489,10 +3287,10 @@
         <v>5</v>
       </c>
       <c r="C11" s="2">
-        <v>9544</v>
+        <v>1518</v>
       </c>
       <c r="D11" s="2">
-        <v>3160</v>
+        <v>2160</v>
       </c>
       <c r="E11" s="2">
         <v>126</v>
@@ -2560,7 +3358,7 @@
         <v>7901</v>
       </c>
       <c r="D15" s="2">
-        <v>2900</v>
+        <v>2935</v>
       </c>
       <c r="E15" s="2">
         <v>104</v>
@@ -2676,7 +3474,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="2">
-        <v>7800</v>
+        <v>7852</v>
       </c>
       <c r="D22" s="2">
         <v>2760</v>
@@ -2863,10 +3661,10 @@
         <v>2</v>
       </c>
       <c r="C33" s="2">
-        <v>7800</v>
+        <v>7789</v>
       </c>
       <c r="D33" s="2">
-        <v>2600</v>
+        <v>2621</v>
       </c>
       <c r="E33" s="2">
         <v>61</v>
@@ -2880,10 +3678,10 @@
         <v>3</v>
       </c>
       <c r="C34" s="2">
-        <v>8900</v>
+        <v>6521</v>
       </c>
       <c r="D34" s="2">
-        <v>3300</v>
+        <v>2935</v>
       </c>
       <c r="E34" s="2">
         <v>85</v>
@@ -2921,6 +3719,261 @@
       </c>
       <c r="E36" s="2">
         <v>115</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B37" s="2">
+        <v>1</v>
+      </c>
+      <c r="C37" s="3">
+        <v>7805</v>
+      </c>
+      <c r="D37" s="3">
+        <v>2859</v>
+      </c>
+      <c r="E37" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B38" s="2">
+        <v>2</v>
+      </c>
+      <c r="C38" s="3">
+        <v>4110</v>
+      </c>
+      <c r="D38" s="3">
+        <v>1572</v>
+      </c>
+      <c r="E38" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B39" s="2">
+        <v>3</v>
+      </c>
+      <c r="C39" s="3">
+        <v>1252</v>
+      </c>
+      <c r="D39" s="3">
+        <v>2317</v>
+      </c>
+      <c r="E39" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B40" s="2">
+        <v>4</v>
+      </c>
+      <c r="C40" s="3">
+        <v>2611</v>
+      </c>
+      <c r="D40" s="3">
+        <v>1201</v>
+      </c>
+      <c r="E40" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B41" s="2">
+        <v>5</v>
+      </c>
+      <c r="C41" s="3">
+        <v>8110</v>
+      </c>
+      <c r="D41" s="3">
+        <v>3116</v>
+      </c>
+      <c r="E41" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B42" s="2">
+        <v>1</v>
+      </c>
+      <c r="C42" s="3">
+        <v>7880</v>
+      </c>
+      <c r="D42" s="3">
+        <v>2860</v>
+      </c>
+      <c r="E42" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B43" s="2">
+        <v>2</v>
+      </c>
+      <c r="C43" s="3">
+        <v>4158</v>
+      </c>
+      <c r="D43" s="3">
+        <v>1515</v>
+      </c>
+      <c r="E43" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44" s="2">
+        <v>3</v>
+      </c>
+      <c r="C44" s="3">
+        <v>2501</v>
+      </c>
+      <c r="D44" s="3">
+        <v>1150</v>
+      </c>
+      <c r="E44" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A45" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B45" s="2">
+        <v>4</v>
+      </c>
+      <c r="C45" s="3">
+        <v>6251</v>
+      </c>
+      <c r="D45" s="3">
+        <v>2751</v>
+      </c>
+      <c r="E45" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B46" s="2">
+        <v>5</v>
+      </c>
+      <c r="C46" s="3">
+        <v>1415</v>
+      </c>
+      <c r="D46" s="3">
+        <v>2151</v>
+      </c>
+      <c r="E46" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B47" s="2">
+        <v>1</v>
+      </c>
+      <c r="C47" s="3">
+        <v>2546</v>
+      </c>
+      <c r="D47" s="3">
+        <v>1321</v>
+      </c>
+      <c r="E47" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B48" s="2">
+        <v>2</v>
+      </c>
+      <c r="C48" s="3">
+        <v>4315</v>
+      </c>
+      <c r="D48" s="3">
+        <v>1560</v>
+      </c>
+      <c r="E48" s="3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B49" s="2">
+        <v>3</v>
+      </c>
+      <c r="C49" s="3">
+        <v>6152</v>
+      </c>
+      <c r="D49" s="3">
+        <v>2553</v>
+      </c>
+      <c r="E49" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B50" s="2">
+        <v>4</v>
+      </c>
+      <c r="C50" s="3">
+        <v>7465</v>
+      </c>
+      <c r="D50" s="3">
+        <v>2821</v>
+      </c>
+      <c r="E50" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B51" s="2">
+        <v>5</v>
+      </c>
+      <c r="C51" s="3">
+        <v>8013</v>
+      </c>
+      <c r="D51" s="3">
+        <v>3017</v>
+      </c>
+      <c r="E51" s="3">
+        <v>100</v>
       </c>
     </row>
   </sheetData>

</xml_diff>